<commit_message>
fullgame/FG-M2: FG2-E2E-01 M2里程碑旅程 账本回写
出口旅程FGJ-M2/FGJ-M2R通过；FG-GAP-050(固件拿不到)、FG-GAP-043(引信固件不可见)
临时打通；新增[M2出口]自检40条。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#CodexEntry-机制图鉴条目.xlsx
+++ b/Configs/GameConfig/Datas/fg/#CodexEntry-机制图鉴条目.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1008,6 +1008,47 @@
         <v>110</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>codex.firmware.restore</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>codex.firmware.restore.title</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>codex.firmware.restore.body</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>codex.firmware.restore.hint</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>codex.firmware.library,codex.signal.raw</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>firmware.restore.first_done</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fullgame/FG-M4: FG4-ECO-06 常驻规则 完成回写账本
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#CodexEntry-机制图鉴条目.xlsx
+++ b/Configs/GameConfig/Datas/fg/#CodexEntry-机制图鉴条目.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1705,6 +1705,47 @@
         <v>270</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>codex.economy.rules</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>codex.economy.rules.title</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>codex.economy.rules.body</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>codex.economy.rules.hint</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>codex.economy.items,codex.build.building</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>rules.panel_first_open,rules.first_created</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>280</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fullgame/FG-M5: FG5-RND-02 解析台 2.0
解析台按身份破解固件/芯片：新增 AnalysisCatalog/AnalysisKind/AnalysisLore 表与
HomeValleyAnalysis.Items；建筑被摧毁（Damaged/Destroyed）时在办项中止、物品退回、
拒收新件；读档对账在办物品按身份不明退回不转废料；旧档解析台入口迁移补测试；
队列芯片完成前核对家园是否仍持有该固件再破解；队列图标不泄露未知物品身份；
被毁/缺件/完成等文案改走文本键。

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#CodexEntry-机制图鉴条目.xlsx
+++ b/Configs/GameConfig/Datas/fg/#CodexEntry-机制图鉴条目.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2033,6 +2033,47 @@
         <v>291</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>codex.research.analysis</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>codex.research.analysis.title</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>codex.research.analysis.body</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>codex.research.analysis.hint</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>codex.research.lab,codex.economy.items</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>analysis.first_enemy_item</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>292</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>